<commit_message>
fix system_prompt_for_integrationTest.md for explicit mock declaration
</commit_message>
<xml_diff>
--- a/gen/finalReport.xlsx
+++ b/gen/finalReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{168AB584-8208-4B92-AE3D-1D90F24B1193}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68400EAE-374C-4FAB-B635-93E5AB146E1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11295" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
   <sheets>
     <sheet name="dolphinscheduler" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="44">
   <si>
     <t>org.apache.dolphinscheduler.api.python.PythonGatewayTest</t>
   </si>
@@ -148,6 +148,30 @@
   </si>
   <si>
     <t>no</t>
+  </si>
+  <si>
+    <t>JUnit import errors</t>
+  </si>
+  <si>
+    <t>Junit import errors</t>
+  </si>
+  <si>
+    <t>com.alibaba.nacos.ai.config.McpConfigurationTest</t>
+  </si>
+  <si>
+    <t>testInit</t>
+  </si>
+  <si>
+    <t>0.008600</t>
+  </si>
+  <si>
+    <t>com.alibaba.nacos.client.naming.remote.http.NamingHttpClientManagerTest</t>
+  </si>
+  <si>
+    <t>testShutdown</t>
+  </si>
+  <si>
+    <t>0.011421</t>
   </si>
 </sst>
 </file>
@@ -524,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B75D52B5-1B5D-406C-B598-869F981E1563}">
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="80" bestFit="1" customWidth="1"/>
@@ -540,13 +564,14 @@
     <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.28515625" customWidth="1"/>
-    <col min="17" max="17" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.28515625" customWidth="1"/>
+    <col min="18" max="18" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -587,19 +612,22 @@
         <v>23</v>
       </c>
       <c r="N1" t="s">
+        <v>37</v>
+      </c>
+      <c r="O1" t="s">
         <v>18</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>28</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -639,20 +667,23 @@
       <c r="M2">
         <v>0</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2">
         <v>22.84</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>16</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -692,20 +723,23 @@
       <c r="M3">
         <v>0</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2">
         <v>18.741</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>16</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>24</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -745,20 +779,23 @@
       <c r="M4">
         <v>0</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2">
         <v>13.975</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>16</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>27</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="R4" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -798,16 +835,19 @@
       <c r="M5">
         <v>0</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5" s="2">
         <v>17.408999999999999</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>16</v>
       </c>
-      <c r="P5" t="s">
+      <c r="Q5" t="s">
         <v>31</v>
       </c>
-      <c r="Q5" t="s">
+      <c r="R5" t="s">
         <v>1</v>
       </c>
     </row>
@@ -819,10 +859,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0CAC5C66-50C3-41AF-881F-738E44943354}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="64.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="71.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" bestFit="1" customWidth="1"/>
@@ -831,16 +871,17 @@
     <col min="7" max="7" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="24.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="24.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="20.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.42578125" customWidth="1"/>
+    <col min="15" max="15" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="8.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>8</v>
       </c>
@@ -881,19 +922,22 @@
         <v>23</v>
       </c>
       <c r="N1" t="s">
+        <v>36</v>
+      </c>
+      <c r="O1" t="s">
         <v>18</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>32</v>
       </c>
@@ -933,20 +977,136 @@
       <c r="M2">
         <v>0</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2">
         <v>13.653</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>16</v>
       </c>
-      <c r="P2" s="1" t="s">
+      <c r="Q2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>0</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3" s="2">
+        <v>13.473000000000001</v>
+      </c>
+      <c r="P3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>40</v>
+      </c>
+      <c r="R3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4" s="2">
+        <v>14.488</v>
+      </c>
+      <c r="P4" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>43</v>
+      </c>
+      <c r="R4" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
added results for AuthHeaderUtilTest
</commit_message>
<xml_diff>
--- a/gen/finalReport.xlsx
+++ b/gen/finalReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAD80AAA-B033-4620-9EBF-0B65166A0091}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E67F08-09F5-430C-BF9E-FC667CCB5E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
+    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="17520" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="62">
   <si>
     <t>org.apache.dolphinscheduler.api.python.PythonGatewayTest</t>
   </si>
@@ -84,12 +84,6 @@
     <t>Generation time (sec)</t>
   </si>
   <si>
-    <t>Argument matchers</t>
-  </si>
-  <si>
-    <t>Transformed argument matchers</t>
-  </si>
-  <si>
     <t>org.apache.dolphinscheduler.api.service.WorkflowTaskLineageServiceTest</t>
   </si>
   <si>
@@ -201,12 +195,6 @@
     <t>Transformed verify with semantic errors</t>
   </si>
   <si>
-    <t>Transformed argument matchers with syntax errors</t>
-  </si>
-  <si>
-    <t>Transformed argument matcher with semantic errors</t>
-  </si>
-  <si>
     <t>Total mocked dependencies</t>
   </si>
   <si>
@@ -214,6 +202,30 @@
   </si>
   <si>
     <t>Transformed verify with syntax errors</t>
+  </si>
+  <si>
+    <t>N.4</t>
+  </si>
+  <si>
+    <t>com.alibaba.nacos.auth.util.AuthHeaderUtilTest</t>
+  </si>
+  <si>
+    <t>testAddIdentityToGrpcRequestWhenNotSupport</t>
+  </si>
+  <si>
+    <t>Argument matchers in thenReturn</t>
+  </si>
+  <si>
+    <t>Transformed argument matchers in thenReturn</t>
+  </si>
+  <si>
+    <t>Transformed argument matchers in thenReturn with syntax errors</t>
+  </si>
+  <si>
+    <t>Transformed argument matcher in thenReturn with semantic errors</t>
+  </si>
+  <si>
+    <t>0.014811</t>
   </si>
 </sst>
 </file>
@@ -607,9 +619,8 @@
   <dimension ref="A1:O24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="48.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="8" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="61.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="23" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="24.42578125" bestFit="1" customWidth="1"/>
@@ -623,7 +634,7 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B1" t="str">
         <f>'TEST IDS'!C2</f>
@@ -653,6 +664,10 @@
         <f>'TEST IDS'!C8</f>
         <v>N.3</v>
       </c>
+      <c r="I1" t="str">
+        <f>'TEST IDS'!C9</f>
+        <v>N.4</v>
+      </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -679,6 +694,9 @@
       <c r="H2">
         <v>0</v>
       </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -706,11 +724,14 @@
       <c r="H3">
         <v>0</v>
       </c>
+      <c r="I3">
+        <v>1</v>
+      </c>
       <c r="O3" s="2"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B4">
         <v>0</v>
@@ -731,13 +752,16 @@
         <v>0</v>
       </c>
       <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
         <v>0</v>
       </c>
       <c r="O4" s="2"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -758,6 +782,9 @@
         <v>0</v>
       </c>
       <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
         <v>0</v>
       </c>
       <c r="O5" s="2"/>
@@ -787,6 +814,9 @@
       <c r="H6">
         <v>1</v>
       </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
       <c r="O6" s="2"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -814,10 +844,13 @@
       <c r="H7">
         <v>1</v>
       </c>
+      <c r="I7">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -838,12 +871,15 @@
         <v>0</v>
       </c>
       <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -864,12 +900,15 @@
         <v>0</v>
       </c>
       <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="B10">
         <v>0</v>
@@ -890,12 +929,15 @@
         <v>0</v>
       </c>
       <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="B11">
         <v>0</v>
@@ -916,12 +958,15 @@
         <v>0</v>
       </c>
       <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -942,12 +987,15 @@
         <v>0</v>
       </c>
       <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B13">
         <v>0</v>
@@ -968,12 +1016,15 @@
         <v>0</v>
       </c>
       <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B14">
         <v>3</v>
@@ -996,10 +1047,13 @@
       <c r="H14">
         <v>1</v>
       </c>
+      <c r="I14">
+        <v>2</v>
+      </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B15">
         <v>0</v>
@@ -1021,6 +1075,9 @@
       </c>
       <c r="H15">
         <v>1</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
@@ -1048,8 +1105,11 @@
       <c r="H16">
         <v>1</v>
       </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>8</v>
       </c>
@@ -1074,8 +1134,11 @@
       <c r="H17">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -1100,10 +1163,13 @@
       <c r="H18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1126,10 +1192,13 @@
       <c r="H19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1152,8 +1221,11 @@
       <c r="H20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>13</v>
       </c>
@@ -1178,10 +1250,13 @@
       <c r="H21" s="2">
         <v>14.488</v>
       </c>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I21" s="2">
+        <v>15.755000000000001</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
         <v>11</v>
@@ -1204,48 +1279,54 @@
       <c r="H22" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I22" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>10</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C23" t="s">
-        <v>19</v>
-      </c>
-      <c r="D23" t="s">
-        <v>22</v>
-      </c>
-      <c r="E23" t="s">
-        <v>26</v>
+      <c r="C23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>24</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G23" t="s">
-        <v>34</v>
-      </c>
-      <c r="H23" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+        <v>27</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E24" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F24" t="s">
         <v>1</v>
@@ -1254,6 +1335,9 @@
         <v>1</v>
       </c>
       <c r="H24" t="s">
+        <v>1</v>
+      </c>
+      <c r="I24" t="s">
         <v>1</v>
       </c>
     </row>
@@ -1265,23 +1349,23 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FEC3C6B7-25E2-4BB7-B16F-5D2201D0E7D7}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="80" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -1292,76 +1376,88 @@
         <v>6</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>54</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
r1 folder for 1st run (not complete)
</commit_message>
<xml_diff>
--- a/gen/finalReport.xlsx
+++ b/gen/finalReport.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedev\Documents\UNICAM\Phd\unmock\gen\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04E67F08-09F5-430C-BF9E-FC667CCB5E17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA18643E-3BBB-4377-B7E6-34C0602D21EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-105" windowWidth="29040" windowHeight="17520" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{398B28D4-6843-470D-81CE-51D800613A8C}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
@@ -1001,7 +1001,7 @@
         <v>0</v>
       </c>
       <c r="C13">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D13">
         <v>0</v>

</xml_diff>